<commit_message>
feat: update gameplay logic
</commit_message>
<xml_diff>
--- a/public/templates/template_import_karyawan.xlsx
+++ b/public/templates/template_import_karyawan.xlsx
@@ -5,24 +5,35 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usman\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usman\OneDrive - Dinas Pendidikan Dan Kebudayaan Kabupaten Lombok Timur\Desktop\mans-cell\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80ABB6A5-D867-41DD-877C-730CC04991F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4E9D95-C9A6-492A-9E1C-E453A47F0551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import Karyawan" sheetId="1" r:id="rId1"/>
     <sheet name="Panduan" sheetId="2" r:id="rId2"/>
     <sheet name="Referensi" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="88">
   <si>
     <t>Sistem Manajemen Karyawan  ·  Isi sesuai format  ·  Jangan ubah nama kolom header</t>
   </si>
@@ -160,6 +171,132 @@
   </si>
   <si>
     <t>Peringgasela</t>
+  </si>
+  <si>
+    <t>RIKA WARDANI</t>
+  </si>
+  <si>
+    <t>Rikawardani593@gmail.com</t>
+  </si>
+  <si>
+    <t>081946324107</t>
+  </si>
+  <si>
+    <t>Karyawan</t>
+  </si>
+  <si>
+    <t>Man'S Cell Sukatain</t>
+  </si>
+  <si>
+    <t>Dusun Repok Baret</t>
+  </si>
+  <si>
+    <t>MIFTAHUL JANNAH</t>
+  </si>
+  <si>
+    <t>Miftahopsi40@gmail.com</t>
+  </si>
+  <si>
+    <t>087882787411</t>
+  </si>
+  <si>
+    <t>Man'S Cell Pringgasela</t>
+  </si>
+  <si>
+    <t>LIDIA FATMI</t>
+  </si>
+  <si>
+    <t>Lidyafatmi0@gmail.com</t>
+  </si>
+  <si>
+    <t>087851370690</t>
+  </si>
+  <si>
+    <t>Dusun Ketembong</t>
+  </si>
+  <si>
+    <t>VINA SABILLA</t>
+  </si>
+  <si>
+    <t>Vinasabilla957@gmail.com</t>
+  </si>
+  <si>
+    <t>087719664066</t>
+  </si>
+  <si>
+    <t>Man'S Cell Pancor</t>
+  </si>
+  <si>
+    <t>Dusun Tanjung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AHMAD ZALDI </t>
+  </si>
+  <si>
+    <t>Bgzalz05@gmail.com</t>
+  </si>
+  <si>
+    <t>083129443582</t>
+  </si>
+  <si>
+    <t>Dusun Danger Masbagik</t>
+  </si>
+  <si>
+    <t>INTAN AZZURA</t>
+  </si>
+  <si>
+    <t>Intanazzura060602@gmail.com</t>
+  </si>
+  <si>
+    <t>087780077562</t>
+  </si>
+  <si>
+    <t>Kepala toko</t>
+  </si>
+  <si>
+    <t>Man'S Cell Aikmel</t>
+  </si>
+  <si>
+    <t>Dusun Pungkang Aikmel</t>
+  </si>
+  <si>
+    <t>RESTIANY</t>
+  </si>
+  <si>
+    <t>Restianyestisny@gmail.com</t>
+  </si>
+  <si>
+    <t>087862251134</t>
+  </si>
+  <si>
+    <t>Dasan Kubur</t>
+  </si>
+  <si>
+    <t>RIADATUSOLIHAN</t>
+  </si>
+  <si>
+    <t>Riadatussolihan@gmail.com</t>
+  </si>
+  <si>
+    <t>087738709028</t>
+  </si>
+  <si>
+    <t>Bpt 02 Cellular</t>
+  </si>
+  <si>
+    <t>ISNAENI MARTHA NINGRUM</t>
+  </si>
+  <si>
+    <t>Isnaenimarthaningrum@gmail.com</t>
+  </si>
+  <si>
+    <t>087763304270</t>
+  </si>
+  <si>
+    <t>Karang Sari</t>
+  </si>
+  <si>
+    <t>AKTIF</t>
   </si>
 </sst>
 </file>
@@ -684,8 +821,8 @@
   <dimension ref="A1:J106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="1" max="1" width="32.42578125" customWidth="1"/>
+    <col min="2" max="2" width="34.42578125" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
@@ -770,7 +907,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="27.95" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>11</v>
       </c>
@@ -803,111 +940,261 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
+      <c r="A7" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="4">
+        <v>2025</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="4">
+        <v>1001</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>87</v>
+      </c>
       <c r="J7" s="4"/>
     </row>
     <row r="8" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
+      <c r="A8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="5">
+        <v>2025</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="5">
+        <v>1002</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>87</v>
+      </c>
       <c r="J8" s="5"/>
     </row>
     <row r="9" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
+      <c r="A9" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D9" s="4">
+        <v>2026</v>
+      </c>
       <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
+      <c r="F9" s="4">
+        <v>1002</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>87</v>
+      </c>
       <c r="J9" s="4"/>
     </row>
     <row r="10" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
+      <c r="A10" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" s="5">
+        <v>2026</v>
+      </c>
       <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
+      <c r="F10" s="5">
+        <v>1003</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>87</v>
+      </c>
       <c r="J10" s="5"/>
     </row>
     <row r="11" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
+      <c r="A11" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" s="4">
+        <v>2025</v>
+      </c>
       <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
+      <c r="F11" s="4">
+        <v>1003</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>87</v>
+      </c>
       <c r="J11" s="4"/>
     </row>
     <row r="12" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
+      <c r="A12" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12" s="5">
+        <v>2023</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" s="5">
+        <v>1004</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>87</v>
+      </c>
       <c r="J12" s="5"/>
     </row>
     <row r="13" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
+      <c r="A13" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13" s="4">
+        <v>2025</v>
+      </c>
       <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
+      <c r="F13" s="4">
+        <v>1004</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>87</v>
+      </c>
       <c r="J13" s="4"/>
     </row>
     <row r="14" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
+      <c r="A14" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="5">
+        <v>2025</v>
+      </c>
       <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
+      <c r="F14" s="5">
+        <v>2001</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>87</v>
+      </c>
       <c r="J14" s="5"/>
     </row>
     <row r="15" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
+      <c r="A15" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D15" s="4">
+        <v>2026</v>
+      </c>
       <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
+      <c r="F15" s="4">
+        <v>2001</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>87</v>
+      </c>
       <c r="J15" s="4"/>
     </row>
     <row r="16" spans="1:10" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>